<commit_message>
Logica de firmas hecha en carpeta con raiz storage/app/public/firmas con nomenclatura del nombre asi (user_id-nombre-apellido)
</commit_message>
<xml_diff>
--- a/storage/app/templates/PLANILLA DE FORMATO DE COMPRA.xlsx
+++ b/storage/app/templates/PLANILLA DE FORMATO DE COMPRA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\SISTEMA-OFICIAL-AGARCORP\storage\app\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Xavier\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E7559D6-3BA5-4768-A3DD-8FF067EBB235}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABACF0F4-D4C9-4884-A184-64D4DE9D5848}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{3208A746-A803-4595-8525-051ED833FA61}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{3208A746-A803-4595-8525-051ED833FA61}"/>
   </bookViews>
   <sheets>
     <sheet name="FORMATO SIN FORMULA" sheetId="2" r:id="rId1"/>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="54">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -207,9 +207,6 @@
   </si>
   <si>
     <t>Solicitado por: {{solicitado_por}}</t>
-  </si>
-  <si>
-    <t>Cargo: {{cargo_solicitante}}</t>
   </si>
   <si>
     <t>Por almacen: {{por_almacen}}</t>
@@ -342,19 +339,28 @@
     <t>{{para_uso_linea3}}</t>
   </si>
   <si>
-    <t>Firma: {{firma_solicitante}}</t>
-  </si>
-  <si>
-    <t>Firma: {{firma_almacen}}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Firma: {{firma_aprobador}}    </t>
-  </si>
-  <si>
-    <t>Firma: {{firma_receptor}}</t>
-  </si>
-  <si>
     <t>{{fecha}}</t>
+  </si>
+  <si>
+    <t>Firma:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cargo: {{cargo_solicitante}} </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> {{firma_solicitante}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Firma: </t>
+  </si>
+  <si>
+    <t>{{firma_almacen}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{{firma_aprobador}}    </t>
+  </si>
+  <si>
+    <t>{{firma_receptor}}</t>
   </si>
 </sst>
 </file>
@@ -1100,6 +1106,166 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="35" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="33" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="34" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="31" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="42" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="29" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1109,30 +1275,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1190,145 +1335,6 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="35" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="33" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="34" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="31" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="42" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="29" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1395,15 +1401,15 @@
       <xdr:twoCellAnchor>
         <xdr:from>
           <xdr:col>2</xdr:col>
-          <xdr:colOff>106680</xdr:colOff>
+          <xdr:colOff>104775</xdr:colOff>
           <xdr:row>26</xdr:row>
-          <xdr:rowOff>129540</xdr:rowOff>
+          <xdr:rowOff>133350</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>4</xdr:col>
-          <xdr:colOff>480060</xdr:colOff>
+          <xdr:colOff>476250</xdr:colOff>
           <xdr:row>26</xdr:row>
-          <xdr:rowOff>129540</xdr:rowOff>
+          <xdr:rowOff>133350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1448,9 +1454,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1488,7 +1494,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1594,7 +1600,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1736,7 +1742,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1748,83 +1754,83 @@
     <tabColor indexed="52"/>
   </sheetPr>
   <dimension ref="C1:N74"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="18" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" style="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5546875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="16.77734375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="11.6640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="18.44140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="16.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="18.42578125" style="1" customWidth="1"/>
     <col min="6" max="6" width="23" style="1" customWidth="1"/>
-    <col min="7" max="7" width="14.88671875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="16.6640625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="24.77734375" style="1" customWidth="1"/>
-    <col min="10" max="10" width="12.6640625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="16.88671875" style="1" customWidth="1"/>
-    <col min="12" max="12" width="14.109375" style="1" customWidth="1"/>
-    <col min="13" max="13" width="21.109375" style="1" customWidth="1"/>
-    <col min="14" max="16384" width="11.44140625" style="1"/>
+    <col min="7" max="7" width="14.85546875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="16.7109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="24.7109375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="16.85546875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="14.140625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="21.140625" style="1" customWidth="1"/>
+    <col min="14" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:13" ht="33.6" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="3:13" ht="18" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="3" spans="3:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="57"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="60" t="s">
+    <row r="1" spans="3:13" ht="33.6" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="3:13" ht="18.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="3:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C3" s="101"/>
+      <c r="D3" s="96"/>
+      <c r="E3" s="104" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="60"/>
-      <c r="G3" s="60"/>
-      <c r="H3" s="60"/>
-      <c r="I3" s="60"/>
-      <c r="J3" s="61"/>
-      <c r="K3" s="66" t="s">
+      <c r="F3" s="104"/>
+      <c r="G3" s="104"/>
+      <c r="H3" s="104"/>
+      <c r="I3" s="104"/>
+      <c r="J3" s="105"/>
+      <c r="K3" s="110" t="s">
         <v>16</v>
       </c>
-      <c r="L3" s="67"/>
-    </row>
-    <row r="4" spans="3:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C4" s="58"/>
-      <c r="D4" s="46"/>
-      <c r="E4" s="62"/>
-      <c r="F4" s="62"/>
-      <c r="G4" s="62"/>
-      <c r="H4" s="62"/>
-      <c r="I4" s="62"/>
-      <c r="J4" s="63"/>
-      <c r="K4" s="68" t="s">
+      <c r="L3" s="111"/>
+    </row>
+    <row r="4" spans="3:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C4" s="102"/>
+      <c r="D4" s="97"/>
+      <c r="E4" s="106"/>
+      <c r="F4" s="106"/>
+      <c r="G4" s="106"/>
+      <c r="H4" s="106"/>
+      <c r="I4" s="106"/>
+      <c r="J4" s="107"/>
+      <c r="K4" s="112" t="s">
         <v>15</v>
       </c>
-      <c r="L4" s="69"/>
-    </row>
-    <row r="5" spans="3:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C5" s="58"/>
-      <c r="D5" s="46"/>
-      <c r="E5" s="62"/>
-      <c r="F5" s="62"/>
-      <c r="G5" s="62"/>
-      <c r="H5" s="62"/>
-      <c r="I5" s="62"/>
-      <c r="J5" s="63"/>
-      <c r="K5" s="68"/>
-      <c r="L5" s="69"/>
-    </row>
-    <row r="6" spans="3:13" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C6" s="59"/>
-      <c r="D6" s="47"/>
-      <c r="E6" s="64"/>
-      <c r="F6" s="64"/>
-      <c r="G6" s="64"/>
-      <c r="H6" s="64"/>
-      <c r="I6" s="64"/>
-      <c r="J6" s="65"/>
-      <c r="K6" s="70" t="s">
+      <c r="L4" s="113"/>
+    </row>
+    <row r="5" spans="3:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C5" s="102"/>
+      <c r="D5" s="97"/>
+      <c r="E5" s="106"/>
+      <c r="F5" s="106"/>
+      <c r="G5" s="106"/>
+      <c r="H5" s="106"/>
+      <c r="I5" s="106"/>
+      <c r="J5" s="107"/>
+      <c r="K5" s="112"/>
+      <c r="L5" s="113"/>
+    </row>
+    <row r="6" spans="3:13" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C6" s="103"/>
+      <c r="D6" s="98"/>
+      <c r="E6" s="108"/>
+      <c r="F6" s="108"/>
+      <c r="G6" s="108"/>
+      <c r="H6" s="108"/>
+      <c r="I6" s="108"/>
+      <c r="J6" s="109"/>
+      <c r="K6" s="114" t="s">
         <v>14</v>
       </c>
-      <c r="L6" s="71"/>
-    </row>
-    <row r="7" spans="3:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L6" s="115"/>
+    </row>
+    <row r="7" spans="3:13" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C7" s="30"/>
       <c r="D7" s="28"/>
       <c r="E7" s="29"/>
@@ -1836,7 +1842,7 @@
       <c r="K7" s="28"/>
       <c r="L7" s="27"/>
     </row>
-    <row r="8" spans="3:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:13" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C8" s="30"/>
       <c r="D8" s="28"/>
       <c r="E8" s="29"/>
@@ -1848,7 +1854,7 @@
       <c r="K8" s="28"/>
       <c r="L8" s="27"/>
     </row>
-    <row r="9" spans="3:13" ht="23.55" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="3:13" ht="23.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C9" s="22"/>
       <c r="D9" s="2"/>
       <c r="E9" s="25" t="s">
@@ -1863,12 +1869,12 @@
       <c r="J9" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="K9" s="118" t="s">
-        <v>51</v>
-      </c>
-      <c r="L9" s="117"/>
-    </row>
-    <row r="10" spans="3:13" ht="23.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K9" s="46" t="s">
+        <v>46</v>
+      </c>
+      <c r="L9" s="45"/>
+    </row>
+    <row r="10" spans="3:13" ht="23.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C10" s="22"/>
       <c r="D10" s="2"/>
       <c r="E10" s="25" t="s">
@@ -1884,7 +1890,7 @@
       <c r="K10" s="24"/>
       <c r="L10" s="23"/>
     </row>
-    <row r="11" spans="3:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="3:13" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C11" s="22"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
@@ -1896,7 +1902,7 @@
       <c r="K11" s="24"/>
       <c r="L11" s="23"/>
     </row>
-    <row r="12" spans="3:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="3:13" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C12" s="22"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
@@ -1908,7 +1914,7 @@
       <c r="K12" s="24"/>
       <c r="L12" s="23"/>
     </row>
-    <row r="13" spans="3:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="3:13" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C13" s="22"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
@@ -1921,34 +1927,34 @@
       <c r="L13" s="21"/>
       <c r="M13" s="2"/>
     </row>
-    <row r="14" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C14" s="92" t="s">
+    <row r="14" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C14" s="56" t="s">
         <v>11</v>
       </c>
-      <c r="D14" s="94" t="s">
+      <c r="D14" s="58" t="s">
         <v>10</v>
       </c>
-      <c r="E14" s="95"/>
-      <c r="F14" s="95"/>
-      <c r="G14" s="95"/>
-      <c r="H14" s="96"/>
-      <c r="I14" s="100" t="s">
+      <c r="E14" s="59"/>
+      <c r="F14" s="59"/>
+      <c r="G14" s="59"/>
+      <c r="H14" s="60"/>
+      <c r="I14" s="64" t="s">
         <v>5</v>
       </c>
-      <c r="J14" s="102" t="s">
+      <c r="J14" s="68" t="s">
         <v>9</v>
       </c>
-      <c r="K14" s="103"/>
-      <c r="L14" s="104"/>
-    </row>
-    <row r="15" spans="3:13" ht="17.55" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C15" s="93"/>
-      <c r="D15" s="97"/>
-      <c r="E15" s="98"/>
-      <c r="F15" s="98"/>
-      <c r="G15" s="98"/>
-      <c r="H15" s="99"/>
-      <c r="I15" s="101"/>
+      <c r="K14" s="69"/>
+      <c r="L14" s="70"/>
+    </row>
+    <row r="15" spans="3:13" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C15" s="57"/>
+      <c r="D15" s="61"/>
+      <c r="E15" s="62"/>
+      <c r="F15" s="62"/>
+      <c r="G15" s="62"/>
+      <c r="H15" s="63"/>
+      <c r="I15" s="65"/>
       <c r="J15" s="20" t="s">
         <v>8</v>
       </c>
@@ -1959,12 +1965,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="3:13" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="3:13" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C16" s="16" t="s">
         <v>27</v>
       </c>
       <c r="D16" s="32" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E16" s="33"/>
       <c r="F16" s="33"/>
@@ -1983,12 +1989,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="3:14" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:14" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C17" s="16" t="s">
         <v>27</v>
       </c>
       <c r="D17" s="32" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E17" s="18"/>
       <c r="F17" s="18"/>
@@ -2007,12 +2013,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C18" s="16" t="s">
         <v>27</v>
       </c>
       <c r="D18" s="32" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E18" s="18"/>
       <c r="F18" s="18"/>
@@ -2031,12 +2037,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C19" s="16" t="s">
         <v>27</v>
       </c>
       <c r="D19" s="32" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E19" s="18"/>
       <c r="F19" s="18"/>
@@ -2055,12 +2061,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="20" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C20" s="16" t="s">
         <v>27</v>
       </c>
       <c r="D20" s="32" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E20" s="18"/>
       <c r="F20" s="18"/>
@@ -2079,12 +2085,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="21" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C21" s="16" t="s">
         <v>27</v>
       </c>
       <c r="D21" s="32" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E21" s="18"/>
       <c r="F21" s="18"/>
@@ -2103,12 +2109,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="22" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C22" s="16" t="s">
         <v>27</v>
       </c>
       <c r="D22" s="32" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E22" s="18"/>
       <c r="F22" s="18"/>
@@ -2127,12 +2133,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="23" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C23" s="16" t="s">
         <v>27</v>
       </c>
       <c r="D23" s="32" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I23" s="35" t="s">
         <v>28</v>
@@ -2147,12 +2153,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="24" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C24" s="16" t="s">
         <v>27</v>
       </c>
       <c r="D24" s="32" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E24" s="40"/>
       <c r="F24" s="40"/>
@@ -2171,12 +2177,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="25" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C25" s="16" t="s">
         <v>27</v>
       </c>
       <c r="D25" s="32" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E25" s="33"/>
       <c r="F25" s="33"/>
@@ -2195,12 +2201,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="26" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C26" s="16" t="s">
         <v>27</v>
       </c>
       <c r="D26" s="32" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E26" s="33"/>
       <c r="F26" s="33"/>
@@ -2219,12 +2225,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C27" s="16" t="s">
         <v>27</v>
       </c>
       <c r="D27" s="32" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E27" s="33"/>
       <c r="F27" s="33"/>
@@ -2243,12 +2249,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C28" s="16" t="s">
         <v>27</v>
       </c>
       <c r="D28" s="32" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E28" s="33"/>
       <c r="F28" s="33"/>
@@ -2267,12 +2273,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C29" s="16" t="s">
         <v>27</v>
       </c>
       <c r="D29" s="32" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E29" s="33"/>
       <c r="F29" s="33"/>
@@ -2291,12 +2297,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="30" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C30" s="16" t="s">
         <v>27</v>
       </c>
       <c r="D30" s="32" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E30" s="33"/>
       <c r="F30" s="33"/>
@@ -2316,7 +2322,7 @@
       </c>
       <c r="N30" s="31"/>
     </row>
-    <row r="31" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C31" s="12"/>
       <c r="D31" s="11"/>
       <c r="E31" s="5"/>
@@ -2328,7 +2334,7 @@
       <c r="K31" s="10"/>
       <c r="L31" s="9"/>
     </row>
-    <row r="32" spans="3:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="3:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C32" s="12"/>
       <c r="D32" s="11"/>
       <c r="E32" s="5"/>
@@ -2340,19 +2346,19 @@
       <c r="K32" s="10"/>
       <c r="L32" s="9"/>
     </row>
-    <row r="33" spans="3:14" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C33" s="115" t="s">
-        <v>44</v>
-      </c>
-      <c r="D33" s="116"/>
-      <c r="E33" s="116"/>
-      <c r="F33" s="116"/>
-      <c r="G33" s="116"/>
-      <c r="H33" s="116"/>
-      <c r="I33" s="116"/>
+    <row r="33" spans="3:14" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C33" s="81" t="s">
+        <v>43</v>
+      </c>
+      <c r="D33" s="82"/>
+      <c r="E33" s="82"/>
+      <c r="F33" s="82"/>
+      <c r="G33" s="82"/>
+      <c r="H33" s="82"/>
+      <c r="I33" s="82"/>
       <c r="L33" s="8"/>
     </row>
-    <row r="34" spans="3:14" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="3:14" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C34" s="36"/>
       <c r="D34" s="37"/>
       <c r="E34" s="37"/>
@@ -2362,65 +2368,65 @@
       <c r="I34" s="37"/>
       <c r="L34" s="8"/>
     </row>
-    <row r="35" spans="3:14" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C35" s="105" t="s">
+    <row r="35" spans="3:14" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C35" s="71" t="s">
         <v>4</v>
       </c>
-      <c r="D35" s="106"/>
-      <c r="E35" s="106"/>
-      <c r="F35" s="77" t="s">
+      <c r="D35" s="72"/>
+      <c r="E35" s="72"/>
+      <c r="F35" s="86" t="s">
         <v>20</v>
       </c>
-      <c r="G35" s="77"/>
+      <c r="G35" s="86"/>
       <c r="H35" s="37"/>
       <c r="I35" s="37"/>
       <c r="L35" s="8"/>
     </row>
-    <row r="36" spans="3:14" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C36" s="105" t="s">
+    <row r="36" spans="3:14" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C36" s="71" t="s">
         <v>3</v>
       </c>
-      <c r="D36" s="106"/>
-      <c r="E36" s="106"/>
-      <c r="F36" s="107" t="s">
+      <c r="D36" s="72"/>
+      <c r="E36" s="72"/>
+      <c r="F36" s="73" t="s">
         <v>21</v>
       </c>
-      <c r="G36" s="107"/>
-      <c r="H36" s="107"/>
-      <c r="I36" s="107"/>
-      <c r="J36" s="107"/>
-      <c r="K36" s="107"/>
-      <c r="L36" s="108"/>
-    </row>
-    <row r="37" spans="3:14" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C37" s="105"/>
-      <c r="D37" s="106"/>
-      <c r="E37" s="106"/>
-      <c r="F37" s="78" t="s">
+      <c r="G36" s="73"/>
+      <c r="H36" s="73"/>
+      <c r="I36" s="73"/>
+      <c r="J36" s="73"/>
+      <c r="K36" s="73"/>
+      <c r="L36" s="74"/>
+    </row>
+    <row r="37" spans="3:14" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C37" s="71"/>
+      <c r="D37" s="72"/>
+      <c r="E37" s="72"/>
+      <c r="F37" s="87" t="s">
         <v>22</v>
       </c>
-      <c r="G37" s="78"/>
-      <c r="H37" s="78"/>
-      <c r="I37" s="78"/>
-      <c r="J37" s="78"/>
-      <c r="K37" s="78"/>
-      <c r="L37" s="79"/>
-    </row>
-    <row r="38" spans="3:14" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C38" s="80"/>
-      <c r="D38" s="81"/>
-      <c r="E38" s="81"/>
-      <c r="F38" s="85" t="s">
-        <v>46</v>
-      </c>
-      <c r="G38" s="85"/>
-      <c r="H38" s="85"/>
-      <c r="I38" s="85"/>
-      <c r="J38" s="85"/>
-      <c r="K38" s="85"/>
-      <c r="L38" s="86"/>
-    </row>
-    <row r="39" spans="3:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G37" s="87"/>
+      <c r="H37" s="87"/>
+      <c r="I37" s="87"/>
+      <c r="J37" s="87"/>
+      <c r="K37" s="87"/>
+      <c r="L37" s="88"/>
+    </row>
+    <row r="38" spans="3:14" ht="34.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C38" s="89"/>
+      <c r="D38" s="90"/>
+      <c r="E38" s="90"/>
+      <c r="F38" s="94" t="s">
+        <v>45</v>
+      </c>
+      <c r="G38" s="94"/>
+      <c r="H38" s="94"/>
+      <c r="I38" s="94"/>
+      <c r="J38" s="94"/>
+      <c r="K38" s="94"/>
+      <c r="L38" s="95"/>
+    </row>
+    <row r="39" spans="3:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C39" s="7"/>
       <c r="D39" s="6"/>
       <c r="E39" s="2"/>
@@ -2432,7 +2438,7 @@
       <c r="K39" s="5"/>
       <c r="L39" s="4"/>
     </row>
-    <row r="40" spans="3:14" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="40" spans="3:14" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C40" s="7"/>
       <c r="D40" s="6"/>
       <c r="E40" s="2"/>
@@ -2445,122 +2451,130 @@
       <c r="L40" s="4"/>
       <c r="N40" s="3"/>
     </row>
-    <row r="41" spans="3:14" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C41" s="75" t="s">
+    <row r="41" spans="3:14" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C41" s="83" t="s">
         <v>23</v>
       </c>
-      <c r="D41" s="55"/>
-      <c r="E41" s="55"/>
-      <c r="F41" s="55"/>
-      <c r="G41" s="76"/>
-      <c r="H41" s="82" t="s">
+      <c r="D41" s="84"/>
+      <c r="E41" s="84"/>
+      <c r="F41" s="84"/>
+      <c r="G41" s="85"/>
+      <c r="H41" s="91" t="s">
         <v>24</v>
       </c>
-      <c r="I41" s="83"/>
-      <c r="J41" s="83"/>
-      <c r="K41" s="83"/>
-      <c r="L41" s="84"/>
-    </row>
-    <row r="42" spans="3:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C42" s="75" t="s">
+      <c r="I41" s="92"/>
+      <c r="J41" s="92"/>
+      <c r="K41" s="92"/>
+      <c r="L41" s="93"/>
+    </row>
+    <row r="42" spans="3:14" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C42" s="83" t="s">
         <v>25</v>
       </c>
-      <c r="D42" s="55"/>
-      <c r="E42" s="55"/>
-      <c r="F42" s="55"/>
-      <c r="G42" s="76"/>
-      <c r="H42" s="54" t="s">
+      <c r="D42" s="84"/>
+      <c r="E42" s="84"/>
+      <c r="F42" s="84"/>
+      <c r="G42" s="85"/>
+      <c r="H42" s="99" t="s">
         <v>26</v>
       </c>
-      <c r="I42" s="55"/>
-      <c r="J42" s="55"/>
-      <c r="K42" s="55"/>
-      <c r="L42" s="56"/>
-    </row>
-    <row r="43" spans="3:14" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C43" s="72" t="s">
+      <c r="I42" s="84"/>
+      <c r="J42" s="84"/>
+      <c r="K42" s="84"/>
+      <c r="L42" s="100"/>
+    </row>
+    <row r="43" spans="3:14" ht="40.15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C43" s="116" t="s">
         <v>32</v>
       </c>
-      <c r="D43" s="73"/>
-      <c r="E43" s="74"/>
-      <c r="F43" s="72" t="s">
+      <c r="D43" s="117"/>
+      <c r="E43" s="118"/>
+      <c r="F43" s="116" t="s">
+        <v>33</v>
+      </c>
+      <c r="G43" s="118"/>
+      <c r="H43" s="116" t="s">
+        <v>35</v>
+      </c>
+      <c r="I43" s="118"/>
+      <c r="J43" s="116" t="s">
+        <v>36</v>
+      </c>
+      <c r="K43" s="117"/>
+      <c r="L43" s="118"/>
+      <c r="N43" s="3"/>
+    </row>
+    <row r="44" spans="3:14" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C44" s="66" t="s">
+        <v>48</v>
+      </c>
+      <c r="D44" s="67"/>
+      <c r="E44" s="47" t="s">
+        <v>49</v>
+      </c>
+      <c r="F44" s="48" t="s">
         <v>34</v>
       </c>
-      <c r="G43" s="74"/>
-      <c r="H43" s="72" t="s">
-        <v>36</v>
-      </c>
-      <c r="I43" s="74"/>
-      <c r="J43" s="72" t="s">
+      <c r="G44" s="50" t="s">
+        <v>51</v>
+      </c>
+      <c r="H44" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="K43" s="73"/>
-      <c r="L43" s="74"/>
-      <c r="N43" s="3"/>
-    </row>
-    <row r="44" spans="3:14" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C44" s="48" t="s">
-        <v>33</v>
-      </c>
-      <c r="D44" s="49"/>
-      <c r="E44" s="50"/>
-      <c r="F44" s="48" t="s">
-        <v>35</v>
-      </c>
-      <c r="G44" s="50"/>
-      <c r="H44" s="48" t="s">
+      <c r="I44" s="50" t="s">
+        <v>52</v>
+      </c>
+      <c r="J44" s="48" t="s">
         <v>38</v>
       </c>
-      <c r="I44" s="50"/>
-      <c r="J44" s="51" t="s">
+      <c r="K44" s="49" t="s">
+        <v>53</v>
+      </c>
+      <c r="L44" s="50"/>
+    </row>
+    <row r="45" spans="3:14" ht="24.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C45" s="75" t="s">
+        <v>47</v>
+      </c>
+      <c r="D45" s="80"/>
+      <c r="E45" s="76"/>
+      <c r="F45" s="75" t="s">
+        <v>50</v>
+      </c>
+      <c r="G45" s="76"/>
+      <c r="H45" s="75" t="s">
+        <v>50</v>
+      </c>
+      <c r="I45" s="76"/>
+      <c r="J45" s="77" t="s">
+        <v>50</v>
+      </c>
+      <c r="K45" s="78"/>
+      <c r="L45" s="79"/>
+    </row>
+    <row r="46" spans="3:14" ht="24.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C46" s="51" t="s">
         <v>39</v>
       </c>
-      <c r="K44" s="52"/>
-      <c r="L44" s="53"/>
-    </row>
-    <row r="45" spans="3:14" ht="24.45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C45" s="109" t="s">
-        <v>47</v>
-      </c>
-      <c r="D45" s="114"/>
-      <c r="E45" s="110"/>
-      <c r="F45" s="109" t="s">
-        <v>48</v>
-      </c>
-      <c r="G45" s="110"/>
-      <c r="H45" s="109" t="s">
-        <v>49</v>
-      </c>
-      <c r="I45" s="110"/>
-      <c r="J45" s="111" t="s">
-        <v>50</v>
-      </c>
-      <c r="K45" s="112"/>
-      <c r="L45" s="113"/>
-    </row>
-    <row r="46" spans="3:14" ht="24.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C46" s="87" t="s">
+      <c r="D46" s="52"/>
+      <c r="E46" s="53"/>
+      <c r="F46" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="D46" s="88"/>
-      <c r="E46" s="89"/>
-      <c r="F46" s="90" t="s">
+      <c r="G46" s="55"/>
+      <c r="H46" s="54" t="s">
         <v>41</v>
       </c>
-      <c r="G46" s="91"/>
-      <c r="H46" s="90" t="s">
+      <c r="I46" s="55"/>
+      <c r="J46" s="38" t="s">
         <v>42</v>
-      </c>
-      <c r="I46" s="91"/>
-      <c r="J46" s="38" t="s">
-        <v>43</v>
       </c>
       <c r="K46" s="39"/>
       <c r="L46" s="42" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="3:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="3:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
       <c r="E47" s="2"/>
@@ -2572,40 +2586,46 @@
       <c r="K47" s="2"/>
       <c r="L47" s="2"/>
     </row>
-    <row r="48" spans="3:14" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="49" spans="13:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="3:14" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="49" spans="13:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="M49" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="13:13" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="51" spans="13:13" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="55" spans="13:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="56" spans="13:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="57" spans="13:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="58" spans="13:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="59" spans="13:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="60" spans="13:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="61" spans="13:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="62" spans="13:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="63" spans="13:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="64" spans="13:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="65" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="66" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="67" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="69" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="71" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="72" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="73" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="74" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="50" spans="13:13" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="51" spans="13:13" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="55" spans="13:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="56" spans="13:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="57" spans="13:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="58" spans="13:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="59" spans="13:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="60" spans="13:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="61" spans="13:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="62" spans="13:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="63" spans="13:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="64" spans="13:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="65" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="66" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="67" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="69" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="71" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="72" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="73" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="74" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="38">
-    <mergeCell ref="C46:E46"/>
-    <mergeCell ref="F46:G46"/>
-    <mergeCell ref="H46:I46"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D14:H15"/>
-    <mergeCell ref="I14:I15"/>
+  <mergeCells count="35">
+    <mergeCell ref="C3:C6"/>
+    <mergeCell ref="E3:J6"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="K6:L6"/>
+    <mergeCell ref="D3:D6"/>
+    <mergeCell ref="H42:L42"/>
+    <mergeCell ref="C43:E43"/>
+    <mergeCell ref="F43:G43"/>
+    <mergeCell ref="H43:I43"/>
+    <mergeCell ref="J43:L43"/>
     <mergeCell ref="J14:L14"/>
     <mergeCell ref="C36:E37"/>
     <mergeCell ref="F36:L36"/>
@@ -2622,22 +2642,13 @@
     <mergeCell ref="C41:G41"/>
     <mergeCell ref="H41:L41"/>
     <mergeCell ref="F38:L38"/>
-    <mergeCell ref="D3:D6"/>
-    <mergeCell ref="C44:E44"/>
-    <mergeCell ref="F44:G44"/>
-    <mergeCell ref="H44:I44"/>
-    <mergeCell ref="J44:L44"/>
-    <mergeCell ref="H42:L42"/>
-    <mergeCell ref="C3:C6"/>
-    <mergeCell ref="E3:J6"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="K6:L6"/>
-    <mergeCell ref="C43:E43"/>
-    <mergeCell ref="F43:G43"/>
-    <mergeCell ref="H43:I43"/>
-    <mergeCell ref="J43:L43"/>
+    <mergeCell ref="C46:E46"/>
+    <mergeCell ref="F46:G46"/>
+    <mergeCell ref="H46:I46"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:H15"/>
+    <mergeCell ref="I14:I15"/>
+    <mergeCell ref="C44:D44"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.23622047244094499" right="0.23622047244094499" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
@@ -2653,15 +2664,15 @@
             <anchor moveWithCells="1" sizeWithCells="1">
               <from>
                 <xdr:col>2</xdr:col>
-                <xdr:colOff>106680</xdr:colOff>
+                <xdr:colOff>104775</xdr:colOff>
                 <xdr:row>26</xdr:row>
-                <xdr:rowOff>129540</xdr:rowOff>
+                <xdr:rowOff>133350</xdr:rowOff>
               </from>
               <to>
                 <xdr:col>4</xdr:col>
-                <xdr:colOff>480060</xdr:colOff>
+                <xdr:colOff>476250</xdr:colOff>
                 <xdr:row>26</xdr:row>
-                <xdr:rowOff>129540</xdr:rowOff>
+                <xdr:rowOff>133350</xdr:rowOff>
               </to>
             </anchor>
           </objectPr>
@@ -2678,7 +2689,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF103C6C-43B0-44D4-BD77-E1E3ABD37B7E}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Correcciones a flujo y a estados
</commit_message>
<xml_diff>
--- a/storage/app/templates/PLANILLA DE FORMATO DE COMPRA.xlsx
+++ b/storage/app/templates/PLANILLA DE FORMATO DE COMPRA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\SISTEMA-OFICIAL-AGARCORP\storage\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43198A9A-0165-4E10-8E0B-E7DF86FB94B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F35CCAA5-D3C8-4F5B-8AF8-4D47EA6205E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{3208A746-A803-4595-8525-051ED833FA61}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{3208A746-A803-4595-8525-051ED833FA61}"/>
   </bookViews>
   <sheets>
     <sheet name="FORMATO SIN FORMULA" sheetId="2" r:id="rId1"/>
@@ -1074,221 +1074,20 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" indent="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" indent="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="39" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="39" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" wrapText="1" indent="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" wrapText="1" indent="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" wrapText="1" indent="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="30" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="28" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="29" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="37" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="38" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="20" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1318,16 +1117,201 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="38" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="30" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="28" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="29" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="37" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="39" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="38" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="20" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" indent="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" indent="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="39" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
@@ -1337,6 +1321,22 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1363,15 +1363,15 @@
       <xdr:twoCellAnchor>
         <xdr:from>
           <xdr:col>2</xdr:col>
-          <xdr:colOff>106680</xdr:colOff>
+          <xdr:colOff>104775</xdr:colOff>
           <xdr:row>26</xdr:row>
-          <xdr:rowOff>137160</xdr:rowOff>
+          <xdr:rowOff>133350</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>4</xdr:col>
-          <xdr:colOff>480060</xdr:colOff>
+          <xdr:colOff>476250</xdr:colOff>
           <xdr:row>26</xdr:row>
-          <xdr:rowOff>137160</xdr:rowOff>
+          <xdr:rowOff>133350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1477,9 +1477,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1517,7 +1517,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1623,7 +1623,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1765,7 +1765,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1777,88 +1777,88 @@
     <tabColor indexed="52"/>
   </sheetPr>
   <dimension ref="B1:O75"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="18" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" style="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5546875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="16.6640625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="11.6640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="18.44140625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="10.21875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="16.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="18.42578125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="11.7109375" style="1" customWidth="1"/>
     <col min="7" max="7" width="10" style="1" customWidth="1"/>
-    <col min="8" max="8" width="16.109375" style="1" customWidth="1"/>
-    <col min="9" max="9" width="12.88671875" style="1" customWidth="1"/>
-    <col min="10" max="10" width="23.21875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="12.6640625" style="1" customWidth="1"/>
-    <col min="12" max="12" width="16.88671875" style="1" customWidth="1"/>
-    <col min="13" max="13" width="14.109375" style="1" customWidth="1"/>
-    <col min="14" max="14" width="21.109375" style="1" customWidth="1"/>
-    <col min="15" max="16384" width="11.44140625" style="1"/>
+    <col min="8" max="8" width="16.140625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="12.85546875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="23.28515625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="12.7109375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="16.85546875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="14.140625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="21.140625" style="1" customWidth="1"/>
+    <col min="15" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:14" ht="33.6" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="3:14" ht="18" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="3" spans="3:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="54"/>
-      <c r="D3" s="69"/>
-      <c r="E3" s="57" t="s">
+    <row r="1" spans="3:14" ht="33.6" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="3:14" ht="18.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="3:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C3" s="102"/>
+      <c r="D3" s="117"/>
+      <c r="E3" s="105" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="58"/>
-      <c r="L3" s="63" t="s">
+      <c r="F3" s="105"/>
+      <c r="G3" s="105"/>
+      <c r="H3" s="105"/>
+      <c r="I3" s="105"/>
+      <c r="J3" s="105"/>
+      <c r="K3" s="106"/>
+      <c r="L3" s="111" t="s">
         <v>15</v>
       </c>
-      <c r="M3" s="64"/>
-    </row>
-    <row r="4" spans="3:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C4" s="55"/>
-      <c r="D4" s="70"/>
-      <c r="E4" s="59"/>
-      <c r="F4" s="59"/>
-      <c r="G4" s="59"/>
-      <c r="H4" s="59"/>
-      <c r="I4" s="59"/>
-      <c r="J4" s="59"/>
-      <c r="K4" s="60"/>
-      <c r="L4" s="65" t="s">
+      <c r="M3" s="112"/>
+    </row>
+    <row r="4" spans="3:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C4" s="103"/>
+      <c r="D4" s="118"/>
+      <c r="E4" s="107"/>
+      <c r="F4" s="107"/>
+      <c r="G4" s="107"/>
+      <c r="H4" s="107"/>
+      <c r="I4" s="107"/>
+      <c r="J4" s="107"/>
+      <c r="K4" s="108"/>
+      <c r="L4" s="113" t="s">
         <v>14</v>
       </c>
-      <c r="M4" s="66"/>
-    </row>
-    <row r="5" spans="3:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C5" s="55"/>
-      <c r="D5" s="70"/>
-      <c r="E5" s="59"/>
-      <c r="F5" s="59"/>
-      <c r="G5" s="59"/>
-      <c r="H5" s="59"/>
-      <c r="I5" s="59"/>
-      <c r="J5" s="59"/>
-      <c r="K5" s="60"/>
-      <c r="L5" s="65"/>
-      <c r="M5" s="66"/>
-    </row>
-    <row r="6" spans="3:14" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C6" s="56"/>
-      <c r="D6" s="71"/>
-      <c r="E6" s="61"/>
-      <c r="F6" s="61"/>
-      <c r="G6" s="61"/>
-      <c r="H6" s="61"/>
-      <c r="I6" s="61"/>
-      <c r="J6" s="61"/>
-      <c r="K6" s="62"/>
-      <c r="L6" s="67" t="s">
+      <c r="M4" s="114"/>
+    </row>
+    <row r="5" spans="3:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C5" s="103"/>
+      <c r="D5" s="118"/>
+      <c r="E5" s="107"/>
+      <c r="F5" s="107"/>
+      <c r="G5" s="107"/>
+      <c r="H5" s="107"/>
+      <c r="I5" s="107"/>
+      <c r="J5" s="107"/>
+      <c r="K5" s="108"/>
+      <c r="L5" s="113"/>
+      <c r="M5" s="114"/>
+    </row>
+    <row r="6" spans="3:14" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C6" s="104"/>
+      <c r="D6" s="119"/>
+      <c r="E6" s="109"/>
+      <c r="F6" s="109"/>
+      <c r="G6" s="109"/>
+      <c r="H6" s="109"/>
+      <c r="I6" s="109"/>
+      <c r="J6" s="109"/>
+      <c r="K6" s="110"/>
+      <c r="L6" s="115" t="s">
         <v>13</v>
       </c>
-      <c r="M6" s="68"/>
-    </row>
-    <row r="7" spans="3:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="M6" s="116"/>
+    </row>
+    <row r="7" spans="3:14" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C7" s="30"/>
       <c r="D7" s="35"/>
       <c r="E7" s="29"/>
@@ -1866,12 +1866,12 @@
       <c r="G7" s="34"/>
       <c r="H7" s="29"/>
       <c r="I7" s="29"/>
-      <c r="J7" s="117"/>
+      <c r="J7" s="53"/>
       <c r="K7" s="29"/>
       <c r="L7" s="35"/>
       <c r="M7" s="20"/>
     </row>
-    <row r="8" spans="3:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:14" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C8" s="31"/>
       <c r="D8" s="35"/>
       <c r="E8" s="29"/>
@@ -1884,16 +1884,16 @@
       <c r="L8" s="35"/>
       <c r="M8" s="20"/>
     </row>
-    <row r="9" spans="3:14" ht="23.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="3:14" ht="23.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C9" s="18"/>
       <c r="D9" s="36"/>
       <c r="E9" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="119" t="s">
+      <c r="F9" s="55" t="s">
         <v>17</v>
       </c>
-      <c r="G9" s="119"/>
+      <c r="G9" s="55"/>
       <c r="H9" s="36"/>
       <c r="I9" s="36"/>
       <c r="J9" s="36"/>
@@ -1905,16 +1905,16 @@
       </c>
       <c r="M9" s="28"/>
     </row>
-    <row r="10" spans="3:14" ht="23.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="3:14" ht="23.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C10" s="46"/>
       <c r="D10" s="36"/>
       <c r="E10" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="118" t="s">
+      <c r="F10" s="54" t="s">
         <v>18</v>
       </c>
-      <c r="G10" s="118"/>
+      <c r="G10" s="54"/>
       <c r="H10" s="36"/>
       <c r="I10" s="36"/>
       <c r="J10" s="36"/>
@@ -1922,7 +1922,7 @@
       <c r="L10" s="40"/>
       <c r="M10" s="19"/>
     </row>
-    <row r="11" spans="3:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="3:14" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C11" s="18"/>
       <c r="D11" s="36"/>
       <c r="E11" s="36"/>
@@ -1935,7 +1935,7 @@
       <c r="L11" s="40"/>
       <c r="M11" s="19"/>
     </row>
-    <row r="12" spans="3:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="3:14" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C12" s="18"/>
       <c r="D12" s="36"/>
       <c r="E12" s="36"/>
@@ -1948,7 +1948,7 @@
       <c r="L12" s="40"/>
       <c r="M12" s="19"/>
     </row>
-    <row r="13" spans="3:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="3:14" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C13" s="47"/>
       <c r="D13" s="36"/>
       <c r="E13" s="36"/>
@@ -1962,36 +1962,36 @@
       <c r="M13" s="17"/>
       <c r="N13" s="2"/>
     </row>
-    <row r="14" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C14" s="95" t="s">
+    <row r="14" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="C14" s="70" t="s">
         <v>10</v>
       </c>
-      <c r="D14" s="97" t="s">
+      <c r="D14" s="72" t="s">
         <v>9</v>
       </c>
-      <c r="E14" s="98"/>
-      <c r="F14" s="98"/>
-      <c r="G14" s="98"/>
-      <c r="H14" s="98"/>
-      <c r="I14" s="99"/>
-      <c r="J14" s="103" t="s">
+      <c r="E14" s="73"/>
+      <c r="F14" s="73"/>
+      <c r="G14" s="73"/>
+      <c r="H14" s="73"/>
+      <c r="I14" s="74"/>
+      <c r="J14" s="78" t="s">
         <v>4</v>
       </c>
-      <c r="K14" s="72" t="s">
+      <c r="K14" s="120" t="s">
         <v>8</v>
       </c>
-      <c r="L14" s="73"/>
-      <c r="M14" s="74"/>
-    </row>
-    <row r="15" spans="3:14" ht="17.7" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C15" s="96"/>
-      <c r="D15" s="100"/>
-      <c r="E15" s="101"/>
-      <c r="F15" s="101"/>
-      <c r="G15" s="101"/>
-      <c r="H15" s="101"/>
-      <c r="I15" s="102"/>
-      <c r="J15" s="104"/>
+      <c r="L14" s="121"/>
+      <c r="M14" s="122"/>
+    </row>
+    <row r="15" spans="3:14" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C15" s="71"/>
+      <c r="D15" s="75"/>
+      <c r="E15" s="76"/>
+      <c r="F15" s="76"/>
+      <c r="G15" s="76"/>
+      <c r="H15" s="76"/>
+      <c r="I15" s="77"/>
+      <c r="J15" s="79"/>
       <c r="K15" s="16" t="s">
         <v>7</v>
       </c>
@@ -2002,7 +2002,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="3:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C16" s="12" t="s">
         <v>26</v>
       </c>
@@ -2027,7 +2027,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="3:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C17" s="12" t="s">
         <v>26</v>
       </c>
@@ -2052,7 +2052,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C18" s="12" t="s">
         <v>26</v>
       </c>
@@ -2077,7 +2077,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="19" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C19" s="12" t="s">
         <v>26</v>
       </c>
@@ -2102,7 +2102,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="20" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C20" s="12" t="s">
         <v>26</v>
       </c>
@@ -2127,7 +2127,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C21" s="12" t="s">
         <v>26</v>
       </c>
@@ -2152,7 +2152,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C22" s="12" t="s">
         <v>26</v>
       </c>
@@ -2177,7 +2177,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C23" s="12" t="s">
         <v>26</v>
       </c>
@@ -2202,7 +2202,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="24" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C24" s="12" t="s">
         <v>26</v>
       </c>
@@ -2227,7 +2227,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="25" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C25" s="12" t="s">
         <v>26</v>
       </c>
@@ -2252,7 +2252,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C26" s="12" t="s">
         <v>26</v>
       </c>
@@ -2277,7 +2277,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="27" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C27" s="12" t="s">
         <v>26</v>
       </c>
@@ -2302,7 +2302,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="28" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C28" s="12" t="s">
         <v>26</v>
       </c>
@@ -2327,7 +2327,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="29" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C29" s="12" t="s">
         <v>26</v>
       </c>
@@ -2352,7 +2352,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="30" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C30" s="12" t="s">
         <v>26</v>
       </c>
@@ -2378,7 +2378,7 @@
       </c>
       <c r="O30" s="21"/>
     </row>
-    <row r="31" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="3:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C31" s="8"/>
       <c r="D31" s="42"/>
       <c r="E31" s="43"/>
@@ -2391,7 +2391,7 @@
       <c r="L31" s="44"/>
       <c r="M31" s="7"/>
     </row>
-    <row r="32" spans="3:15" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="3:15" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C32" s="8"/>
       <c r="D32" s="42"/>
       <c r="E32" s="43"/>
@@ -2404,22 +2404,22 @@
       <c r="L32" s="44"/>
       <c r="M32" s="7"/>
     </row>
-    <row r="33" spans="2:15" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C33" s="79" t="s">
+    <row r="33" spans="2:15" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C33" s="87" t="s">
         <v>41</v>
       </c>
-      <c r="D33" s="80"/>
-      <c r="E33" s="80"/>
-      <c r="F33" s="80"/>
-      <c r="G33" s="80"/>
-      <c r="H33" s="80"/>
-      <c r="I33" s="80"/>
-      <c r="J33" s="80"/>
+      <c r="D33" s="88"/>
+      <c r="E33" s="88"/>
+      <c r="F33" s="88"/>
+      <c r="G33" s="88"/>
+      <c r="H33" s="88"/>
+      <c r="I33" s="88"/>
+      <c r="J33" s="88"/>
       <c r="K33" s="41"/>
       <c r="L33" s="41"/>
       <c r="M33" s="6"/>
     </row>
-    <row r="34" spans="2:15" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:15" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C34" s="32"/>
       <c r="D34" s="33"/>
       <c r="E34" s="33"/>
@@ -2432,71 +2432,71 @@
       <c r="L34" s="41"/>
       <c r="M34" s="6"/>
     </row>
-    <row r="35" spans="2:15" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C35" s="75" t="s">
+    <row r="35" spans="2:15" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C35" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="D35" s="76"/>
-      <c r="E35" s="76"/>
-      <c r="F35" s="82" t="s">
+      <c r="D35" s="90"/>
+      <c r="E35" s="90"/>
+      <c r="F35" s="91" t="s">
         <v>19</v>
       </c>
-      <c r="G35" s="82"/>
-      <c r="H35" s="82"/>
+      <c r="G35" s="91"/>
+      <c r="H35" s="91"/>
       <c r="I35" s="33"/>
       <c r="J35" s="33"/>
       <c r="K35" s="41"/>
       <c r="L35" s="41"/>
       <c r="M35" s="6"/>
     </row>
-    <row r="36" spans="2:15" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C36" s="75" t="s">
+    <row r="36" spans="2:15" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C36" s="89" t="s">
         <v>2</v>
       </c>
-      <c r="D36" s="76"/>
-      <c r="E36" s="76"/>
-      <c r="F36" s="77" t="s">
+      <c r="D36" s="90"/>
+      <c r="E36" s="90"/>
+      <c r="F36" s="123" t="s">
         <v>20</v>
       </c>
-      <c r="G36" s="77"/>
-      <c r="H36" s="77"/>
-      <c r="I36" s="77"/>
-      <c r="J36" s="77"/>
-      <c r="K36" s="77"/>
-      <c r="L36" s="77"/>
-      <c r="M36" s="78"/>
-    </row>
-    <row r="37" spans="2:15" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C37" s="75"/>
-      <c r="D37" s="76"/>
-      <c r="E37" s="76"/>
-      <c r="F37" s="83" t="s">
+      <c r="G36" s="123"/>
+      <c r="H36" s="123"/>
+      <c r="I36" s="123"/>
+      <c r="J36" s="123"/>
+      <c r="K36" s="123"/>
+      <c r="L36" s="123"/>
+      <c r="M36" s="124"/>
+    </row>
+    <row r="37" spans="2:15" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C37" s="89"/>
+      <c r="D37" s="90"/>
+      <c r="E37" s="90"/>
+      <c r="F37" s="92" t="s">
         <v>21</v>
       </c>
-      <c r="G37" s="83"/>
-      <c r="H37" s="83"/>
-      <c r="I37" s="83"/>
-      <c r="J37" s="83"/>
-      <c r="K37" s="83"/>
-      <c r="L37" s="83"/>
-      <c r="M37" s="84"/>
-    </row>
-    <row r="38" spans="2:15" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C38" s="85"/>
-      <c r="D38" s="86"/>
-      <c r="E38" s="86"/>
-      <c r="F38" s="88" t="s">
+      <c r="G37" s="92"/>
+      <c r="H37" s="92"/>
+      <c r="I37" s="92"/>
+      <c r="J37" s="92"/>
+      <c r="K37" s="92"/>
+      <c r="L37" s="92"/>
+      <c r="M37" s="93"/>
+    </row>
+    <row r="38" spans="2:15" ht="34.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C38" s="94"/>
+      <c r="D38" s="95"/>
+      <c r="E38" s="95"/>
+      <c r="F38" s="97" t="s">
         <v>43</v>
       </c>
-      <c r="G38" s="88"/>
-      <c r="H38" s="88"/>
-      <c r="I38" s="88"/>
-      <c r="J38" s="88"/>
-      <c r="K38" s="88"/>
-      <c r="L38" s="88"/>
-      <c r="M38" s="89"/>
-    </row>
-    <row r="39" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G38" s="97"/>
+      <c r="H38" s="97"/>
+      <c r="I38" s="97"/>
+      <c r="J38" s="97"/>
+      <c r="K38" s="97"/>
+      <c r="L38" s="97"/>
+      <c r="M38" s="98"/>
+    </row>
+    <row r="39" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C39" s="5"/>
       <c r="D39" s="45"/>
       <c r="E39" s="36"/>
@@ -2509,7 +2509,7 @@
       <c r="L39" s="43"/>
       <c r="M39" s="4"/>
     </row>
-    <row r="40" spans="2:15" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="40" spans="2:15" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C40" s="5"/>
       <c r="D40" s="45"/>
       <c r="E40" s="36"/>
@@ -2523,147 +2523,147 @@
       <c r="M40" s="4"/>
       <c r="O40" s="3"/>
     </row>
-    <row r="41" spans="2:15" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C41" s="81" t="s">
+    <row r="41" spans="2:15" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C41" s="80" t="s">
         <v>22</v>
       </c>
-      <c r="D41" s="81"/>
-      <c r="E41" s="81"/>
-      <c r="F41" s="81"/>
-      <c r="G41" s="81"/>
-      <c r="H41" s="81"/>
-      <c r="I41" s="87" t="s">
+      <c r="D41" s="80"/>
+      <c r="E41" s="80"/>
+      <c r="F41" s="80"/>
+      <c r="G41" s="80"/>
+      <c r="H41" s="80"/>
+      <c r="I41" s="96" t="s">
         <v>23</v>
       </c>
-      <c r="J41" s="87"/>
-      <c r="K41" s="87"/>
-      <c r="L41" s="87"/>
-      <c r="M41" s="87"/>
-    </row>
-    <row r="42" spans="2:15" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C42" s="81" t="s">
+      <c r="J41" s="96"/>
+      <c r="K41" s="96"/>
+      <c r="L41" s="96"/>
+      <c r="M41" s="96"/>
+    </row>
+    <row r="42" spans="2:15" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C42" s="80" t="s">
         <v>24</v>
       </c>
-      <c r="D42" s="81"/>
-      <c r="E42" s="81"/>
-      <c r="F42" s="81"/>
-      <c r="G42" s="81"/>
-      <c r="H42" s="81"/>
-      <c r="I42" s="81" t="s">
+      <c r="D42" s="80"/>
+      <c r="E42" s="80"/>
+      <c r="F42" s="80"/>
+      <c r="G42" s="80"/>
+      <c r="H42" s="80"/>
+      <c r="I42" s="80" t="s">
         <v>25</v>
       </c>
-      <c r="J42" s="81"/>
-      <c r="K42" s="81"/>
-      <c r="L42" s="81"/>
-      <c r="M42" s="81"/>
-    </row>
-    <row r="43" spans="2:15" ht="40.200000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C43" s="105" t="s">
+      <c r="J42" s="80"/>
+      <c r="K42" s="80"/>
+      <c r="L42" s="80"/>
+      <c r="M42" s="80"/>
+    </row>
+    <row r="43" spans="2:15" ht="40.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C43" s="81" t="s">
         <v>31</v>
       </c>
-      <c r="D43" s="106"/>
-      <c r="E43" s="107"/>
-      <c r="F43" s="105" t="s">
+      <c r="D43" s="82"/>
+      <c r="E43" s="83"/>
+      <c r="F43" s="81" t="s">
         <v>32</v>
       </c>
-      <c r="G43" s="106"/>
-      <c r="H43" s="107"/>
-      <c r="I43" s="105" t="s">
+      <c r="G43" s="82"/>
+      <c r="H43" s="83"/>
+      <c r="I43" s="81" t="s">
         <v>34</v>
       </c>
-      <c r="J43" s="107"/>
-      <c r="K43" s="105" t="s">
+      <c r="J43" s="83"/>
+      <c r="K43" s="81" t="s">
         <v>35</v>
       </c>
-      <c r="L43" s="106"/>
-      <c r="M43" s="107"/>
+      <c r="L43" s="82"/>
+      <c r="M43" s="83"/>
       <c r="O43" s="3"/>
     </row>
-    <row r="44" spans="2:15" ht="25.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C44" s="48" t="s">
+    <row r="44" spans="2:15" ht="25.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C44" s="84" t="s">
         <v>45</v>
       </c>
-      <c r="D44" s="49"/>
-      <c r="E44" s="50"/>
-      <c r="F44" s="48" t="s">
+      <c r="D44" s="86"/>
+      <c r="E44" s="85"/>
+      <c r="F44" s="84" t="s">
         <v>33</v>
       </c>
-      <c r="G44" s="49"/>
-      <c r="H44" s="50"/>
-      <c r="I44" s="48" t="s">
+      <c r="G44" s="86"/>
+      <c r="H44" s="85"/>
+      <c r="I44" s="84" t="s">
         <v>36</v>
       </c>
-      <c r="J44" s="50"/>
-      <c r="K44" s="48" t="s">
+      <c r="J44" s="85"/>
+      <c r="K44" s="84" t="s">
         <v>37</v>
       </c>
-      <c r="L44" s="49"/>
-      <c r="M44" s="50"/>
-    </row>
-    <row r="45" spans="2:15" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C45" s="111"/>
-      <c r="D45" s="123" t="s">
+      <c r="L44" s="86"/>
+      <c r="M44" s="85"/>
+    </row>
+    <row r="45" spans="2:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C45" s="48"/>
+      <c r="D45" s="59" t="s">
         <v>50</v>
       </c>
-      <c r="E45" s="124"/>
-      <c r="F45" s="120"/>
-      <c r="G45" s="121" t="s">
+      <c r="E45" s="60"/>
+      <c r="F45" s="56"/>
+      <c r="G45" s="57" t="s">
         <v>47</v>
       </c>
-      <c r="H45" s="122"/>
-      <c r="I45" s="125"/>
-      <c r="J45" s="127" t="s">
+      <c r="H45" s="58"/>
+      <c r="I45" s="61"/>
+      <c r="J45" s="132" t="s">
         <v>48</v>
       </c>
-      <c r="K45" s="128"/>
-      <c r="L45" s="126" t="s">
+      <c r="K45" s="63"/>
+      <c r="L45" s="62" t="s">
         <v>49</v>
       </c>
-      <c r="M45" s="112"/>
-    </row>
-    <row r="46" spans="2:15" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C46" s="108" t="s">
+      <c r="M45" s="49"/>
+    </row>
+    <row r="46" spans="2:15" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C46" s="128" t="s">
         <v>44</v>
       </c>
-      <c r="D46" s="109"/>
-      <c r="E46" s="110"/>
-      <c r="F46" s="113" t="s">
+      <c r="D46" s="129"/>
+      <c r="E46" s="130"/>
+      <c r="F46" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="G46" s="115"/>
-      <c r="H46" s="114"/>
-      <c r="I46" s="113" t="s">
+      <c r="G46" s="52"/>
+      <c r="H46" s="51"/>
+      <c r="I46" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="J46" s="129"/>
-      <c r="K46" s="130" t="s">
+      <c r="J46" s="131"/>
+      <c r="K46" s="125" t="s">
         <v>46</v>
       </c>
-      <c r="L46" s="131"/>
-      <c r="M46" s="132"/>
-    </row>
-    <row r="47" spans="2:15" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C47" s="90" t="s">
+      <c r="L46" s="126"/>
+      <c r="M46" s="127"/>
+    </row>
+    <row r="47" spans="2:15" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C47" s="64" t="s">
         <v>38</v>
       </c>
-      <c r="D47" s="91"/>
-      <c r="E47" s="92"/>
-      <c r="F47" s="93" t="s">
+      <c r="D47" s="65"/>
+      <c r="E47" s="66"/>
+      <c r="F47" s="67" t="s">
         <v>39</v>
       </c>
-      <c r="G47" s="116"/>
-      <c r="H47" s="94"/>
-      <c r="I47" s="93" t="s">
+      <c r="G47" s="68"/>
+      <c r="H47" s="69"/>
+      <c r="I47" s="67" t="s">
         <v>40</v>
       </c>
-      <c r="J47" s="94"/>
-      <c r="K47" s="51" t="s">
+      <c r="J47" s="69"/>
+      <c r="K47" s="99" t="s">
         <v>52</v>
       </c>
-      <c r="L47" s="52"/>
-      <c r="M47" s="53"/>
-    </row>
-    <row r="48" spans="2:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L47" s="100"/>
+      <c r="M47" s="101"/>
+    </row>
+    <row r="48" spans="2:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B48" s="21"/>
       <c r="C48" s="36"/>
       <c r="D48" s="36"/>
@@ -2677,7 +2677,7 @@
       <c r="L48" s="36"/>
       <c r="M48" s="36"/>
     </row>
-    <row r="49" spans="3:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="3:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C49" s="41"/>
       <c r="D49" s="41"/>
       <c r="E49" s="41"/>
@@ -2690,35 +2690,56 @@
       <c r="L49" s="41"/>
       <c r="M49" s="41"/>
     </row>
-    <row r="50" spans="3:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="3:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="N50" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="3:14" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="52" spans="3:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="3:14" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="52" spans="3:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="H52" s="21"/>
     </row>
-    <row r="56" spans="3:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="57" spans="3:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="58" spans="3:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="59" spans="3:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="60" spans="3:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="61" spans="3:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="62" spans="3:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="63" spans="3:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="64" spans="3:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="65" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="66" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="67" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="68" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="70" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="72" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="73" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="74" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="75" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="56" spans="3:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="57" spans="3:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="58" spans="3:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="59" spans="3:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="60" spans="3:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="61" spans="3:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="62" spans="3:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="63" spans="3:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="64" spans="3:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="65" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="66" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="67" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="68" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="70" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="72" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="73" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="74" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="75" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="37">
+    <mergeCell ref="K44:M44"/>
+    <mergeCell ref="K47:M47"/>
+    <mergeCell ref="C3:C6"/>
+    <mergeCell ref="E3:K6"/>
+    <mergeCell ref="L3:M3"/>
+    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="L6:M6"/>
+    <mergeCell ref="D3:D6"/>
+    <mergeCell ref="K14:M14"/>
+    <mergeCell ref="C36:E37"/>
+    <mergeCell ref="F36:M36"/>
+    <mergeCell ref="K46:M46"/>
+    <mergeCell ref="C46:E46"/>
+    <mergeCell ref="C42:H42"/>
+    <mergeCell ref="F35:H35"/>
+    <mergeCell ref="F37:M37"/>
+    <mergeCell ref="C38:E38"/>
+    <mergeCell ref="C41:H41"/>
+    <mergeCell ref="I41:M41"/>
+    <mergeCell ref="F38:M38"/>
     <mergeCell ref="C47:E47"/>
     <mergeCell ref="F47:H47"/>
     <mergeCell ref="I47:J47"/>
@@ -2735,27 +2756,6 @@
     <mergeCell ref="F44:H44"/>
     <mergeCell ref="C33:J33"/>
     <mergeCell ref="C35:E35"/>
-    <mergeCell ref="C42:H42"/>
-    <mergeCell ref="F35:H35"/>
-    <mergeCell ref="F37:M37"/>
-    <mergeCell ref="C38:E38"/>
-    <mergeCell ref="C41:H41"/>
-    <mergeCell ref="I41:M41"/>
-    <mergeCell ref="F38:M38"/>
-    <mergeCell ref="K44:M44"/>
-    <mergeCell ref="K47:M47"/>
-    <mergeCell ref="C3:C6"/>
-    <mergeCell ref="E3:K6"/>
-    <mergeCell ref="L3:M3"/>
-    <mergeCell ref="L4:M4"/>
-    <mergeCell ref="L5:M5"/>
-    <mergeCell ref="L6:M6"/>
-    <mergeCell ref="D3:D6"/>
-    <mergeCell ref="K14:M14"/>
-    <mergeCell ref="C36:E37"/>
-    <mergeCell ref="F36:M36"/>
-    <mergeCell ref="K46:M46"/>
-    <mergeCell ref="C46:E46"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.23622047244094499" right="0.23622047244094499" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
@@ -2771,15 +2771,15 @@
             <anchor moveWithCells="1" sizeWithCells="1">
               <from>
                 <xdr:col>2</xdr:col>
-                <xdr:colOff>106680</xdr:colOff>
+                <xdr:colOff>104775</xdr:colOff>
                 <xdr:row>26</xdr:row>
-                <xdr:rowOff>137160</xdr:rowOff>
+                <xdr:rowOff>133350</xdr:rowOff>
               </from>
               <to>
                 <xdr:col>4</xdr:col>
-                <xdr:colOff>480060</xdr:colOff>
+                <xdr:colOff>476250</xdr:colOff>
                 <xdr:row>26</xdr:row>
-                <xdr:rowOff>137160</xdr:rowOff>
+                <xdr:rowOff>133350</xdr:rowOff>
               </to>
             </anchor>
           </objectPr>
@@ -2796,7 +2796,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF103C6C-43B0-44D4-BD77-E1E3ABD37B7E}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>